<commit_message>
feat: add folder images
</commit_message>
<xml_diff>
--- a/dataset/teste.xlsx
+++ b/dataset/teste.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,127 +424,72 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>23/07/2026</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>20/07/2026</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>19/07/2026</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>17/07/2026</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>15/07/2026</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>14/07/2026</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>13/07/2026</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>12/07/2026</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>10/07/2026</t>
-        </is>
-      </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>05/07/2026</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>03/07/2026</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>30/06/2026</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>29/06/2026</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
           <t>18/07/2026</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>11/07/2026</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>04/07/2026</t>
         </is>
       </c>
     </row>
@@ -558,74 +503,43 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5.77367</v>
+        <v>5.83771</v>
       </c>
       <c r="D2" t="n">
+        <v>5.82411</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5.78369</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5.7971</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5.79039</v>
+      </c>
+      <c r="H2" t="n">
         <v>5.78035</v>
       </c>
-      <c r="E2" t="n">
+      <c r="I2" t="n">
         <v>5.79374</v>
       </c>
-      <c r="F2" t="n">
+      <c r="J2" t="n">
         <v>5.82072</v>
       </c>
-      <c r="G2" t="n">
+      <c r="K2" t="n">
         <v>5.8548</v>
       </c>
-      <c r="H2" t="n">
+      <c r="L2" t="n">
         <v>5.86167</v>
       </c>
-      <c r="I2" t="n">
+      <c r="M2" t="n">
         <v>5.84454</v>
       </c>
-      <c r="J2" t="n">
+      <c r="N2" t="n">
         <v>5.83771</v>
       </c>
-      <c r="K2" t="n">
-        <v>5.80383</v>
-      </c>
-      <c r="L2" t="n">
-        <v>5.8548</v>
-      </c>
-      <c r="M2" t="n">
-        <v>5.82072</v>
-      </c>
-      <c r="N2" t="n">
-        <v>5.84454</v>
-      </c>
-      <c r="O2" t="n">
-        <v>5.86855</v>
-      </c>
-      <c r="P2" t="n">
-        <v>5.89275</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>5.89275</v>
-      </c>
-      <c r="R2" t="n">
-        <v>5.8789</v>
-      </c>
-      <c r="S2" t="n">
-        <v>5.92417</v>
-      </c>
-      <c r="T2" t="n">
-        <v>5.92768</v>
-      </c>
-      <c r="U2" t="n">
-        <v>5.95948</v>
-      </c>
-      <c r="V2" t="n">
-        <v>5.92768</v>
-      </c>
-      <c r="W2" t="n">
-        <v>5.90319</v>
-      </c>
-      <c r="X2" t="n">
-        <v>5.92066</v>
-      </c>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -637,74 +551,43 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5.0546</v>
+        <v>5.137</v>
       </c>
       <c r="D3" t="n">
+        <v>5.1286</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5.0825</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.0785</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5.097</v>
+      </c>
+      <c r="H3" t="n">
         <v>5.06537</v>
       </c>
-      <c r="E3" t="n">
+      <c r="I3" t="n">
         <v>5.0877</v>
       </c>
-      <c r="F3" t="n">
+      <c r="J3" t="n">
         <v>5.1051</v>
       </c>
-      <c r="G3" t="n">
+      <c r="K3" t="n">
         <v>5.1207</v>
       </c>
-      <c r="H3" t="n">
+      <c r="L3" t="n">
         <v>5.1047</v>
       </c>
-      <c r="I3" t="n">
+      <c r="M3" t="n">
         <v>5.1139</v>
       </c>
-      <c r="J3" t="n">
+      <c r="N3" t="n">
         <v>5.0908</v>
       </c>
-      <c r="K3" t="n">
-        <v>5.088</v>
-      </c>
-      <c r="L3" t="n">
-        <v>5.148</v>
-      </c>
-      <c r="M3" t="n">
-        <v>5.1079</v>
-      </c>
-      <c r="N3" t="n">
-        <v>5.1064</v>
-      </c>
-      <c r="O3" t="n">
-        <v>5.1339</v>
-      </c>
-      <c r="P3" t="n">
-        <v>5.1631</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>5.1709</v>
-      </c>
-      <c r="R3" t="n">
-        <v>5.1436</v>
-      </c>
-      <c r="S3" t="n">
-        <v>5.1844</v>
-      </c>
-      <c r="T3" t="n">
-        <v>5.165</v>
-      </c>
-      <c r="U3" t="n">
-        <v>5.222</v>
-      </c>
-      <c r="V3" t="n">
-        <v>5.2206</v>
-      </c>
-      <c r="W3" t="n">
-        <v>5.1746</v>
-      </c>
-      <c r="X3" t="n">
-        <v>5.1874</v>
-      </c>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -716,73 +599,42 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>333698</v>
+        <v>328662</v>
       </c>
       <c r="D4" t="n">
+        <v>326961</v>
+      </c>
+      <c r="E4" t="n">
+        <v>333641</v>
+      </c>
+      <c r="F4" t="n">
+        <v>327902</v>
+      </c>
+      <c r="G4" t="n">
+        <v>332610</v>
+      </c>
+      <c r="H4" t="n">
         <v>336308</v>
       </c>
-      <c r="E4" t="n">
+      <c r="I4" t="n">
         <v>339276</v>
       </c>
-      <c r="F4" t="n">
+      <c r="J4" t="n">
         <v>334324</v>
       </c>
-      <c r="G4" t="n">
+      <c r="K4" t="n">
         <v>332990</v>
       </c>
-      <c r="H4" t="n">
+      <c r="L4" t="n">
         <v>329036</v>
       </c>
-      <c r="I4" t="n">
-        <v>327720</v>
-      </c>
-      <c r="J4" t="n">
-        <v>330996</v>
-      </c>
-      <c r="K4" t="n">
-        <v>332241</v>
-      </c>
-      <c r="L4" t="n">
-        <v>322439</v>
-      </c>
-      <c r="M4" t="n">
-        <v>328600</v>
-      </c>
-      <c r="N4" t="n">
-        <v>330624</v>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>326167</v>
+        <v>328854</v>
       </c>
       <c r="P4" t="n">
-        <v>324355</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>331470</v>
-      </c>
-      <c r="R4" t="n">
-        <v>334353</v>
-      </c>
-      <c r="S4" t="n">
-        <v>335454</v>
-      </c>
-      <c r="T4" t="n">
-        <v>331041</v>
-      </c>
-      <c r="U4" t="n">
-        <v>323748</v>
-      </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="n">
         <v>334000</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>329289</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>332885</v>
       </c>
     </row>
   </sheetData>

</xml_diff>